<commit_message>
wip snapshot from Chaos at 2026-10-07T11:55:58-04:00 (not a real commit; resume with tools/sync.py wip)
</commit_message>
<xml_diff>
--- a/Beelzebub/Beelzebub/docs/V0136_ABILITY_TEST_PLAN.xlsx
+++ b/Beelzebub/Beelzebub/docs/V0136_ABILITY_TEST_PLAN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13344a214c4487a6/Documents/CURSOR PROJECTS/Games/V Rising/Beelzebub Lord of Gluttony/Beelzebub/Beelzebub/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_0C8F69643AC9C97A0A4CDA8E81F44656D995E8B5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_0C8F69643AC9C97A0A4CDA8E81F44656D995E8B5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CD5E864-CBA7-490C-93E6-0FAB72414583}"/>
   <bookViews>
-    <workbookView xWindow="15705" yWindow="3945" windowWidth="32145" windowHeight="15345" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start here" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3974" uniqueCount="2323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3982" uniqueCount="2326">
   <si>
     <t>Beelzebub v0.136 — ability test plan</t>
   </si>
@@ -8131,6 +8131,15 @@
   </si>
   <si>
     <t>Doesn't drop from this unit by default. `.beelz admin ability AB_Wolf_Boss_DashAttack_Double_AbilityGroup` shows enabled=off. Re-enable with `.beelz admin ability AB_Wolf_Boss_DashAttack_Double_AbilityGroup enabled true`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Works with 120 second cooldown </t>
+  </si>
+  <si>
+    <t>Works with 3 sec shortened cooldown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Works with 10 second cooldown.  However, notably there are two of this ability.  Only one gained the cooldown.  Also notably the other without the cooldown is a chain attack.  There are two attacks in the series, each of which is triggered via button push.  I don't know if the one with a cooldown was the same.  </t>
   </si>
 </sst>
 </file>
@@ -8841,7 +8850,7 @@
       </c>
       <c r="C6" s="6">
         <f>COUNTIF(Presets!L2:L210,"Pass")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D6" s="7">
         <f>COUNTIF(Presets!L2:L210,"Partial")</f>
@@ -8857,7 +8866,7 @@
       </c>
       <c r="G6" s="10">
         <f>IF(B6=0,0,SUM(C6:F6)/B6)</f>
-        <v>0</v>
+        <v>1.9138755980861243E-2</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -8926,7 +8935,7 @@
       </c>
       <c r="C9" s="13">
         <f>SUM(C6:C8)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D9" s="14">
         <f>SUM(D6:D8)</f>
@@ -8942,7 +8951,7 @@
       </c>
       <c r="G9" s="10">
         <f>IF(B9=0,0,SUM(C9:F9)/B9)</f>
-        <v>0</v>
+        <v>6.5040650406504065E-3</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
@@ -9255,8 +9264,12 @@
       <c r="J2" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="K2" s="20"/>
-      <c r="L2" s="21"/>
+      <c r="K2" s="20" t="s">
+        <v>2323</v>
+      </c>
+      <c r="L2" s="21" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" spans="1:12" ht="78.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
@@ -9289,8 +9302,12 @@
       <c r="J3" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="21"/>
+      <c r="K3" s="20" t="s">
+        <v>2323</v>
+      </c>
+      <c r="L3" s="21" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" spans="1:12" ht="78.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
@@ -9323,8 +9340,12 @@
       <c r="J4" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="K4" s="20"/>
-      <c r="L4" s="21"/>
+      <c r="K4" s="20" t="s">
+        <v>2324</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" spans="1:12" ht="108.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
@@ -9357,8 +9378,12 @@
       <c r="J5" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="K5" s="20"/>
-      <c r="L5" s="21"/>
+      <c r="K5" s="20" t="s">
+        <v>2325</v>
+      </c>
+      <c r="L5" s="21" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="6" spans="1:12" ht="78.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5">

</xml_diff>

<commit_message>
wip snapshot from Chaos at 2026-10-15T12:29:21-04:00 (not a real commit; resume with tools/sync.py wip)
</commit_message>
<xml_diff>
--- a/Beelzebub/Beelzebub/docs/V0136_ABILITY_TEST_PLAN.xlsx
+++ b/Beelzebub/Beelzebub/docs/V0136_ABILITY_TEST_PLAN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13344a214c4487a6/Documents/CURSOR PROJECTS/Games/V Rising/Beelzebub Lord of Gluttony/Beelzebub/Beelzebub/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_0C8F69643AC9C97A0A4CDA8E81F44656D995E8B5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_0C8F69643AC9C97A0A4CDA8E81F44656D995E8B5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3CD5E864-CBA7-490C-93E6-0FAB72414583}"/>
   <bookViews>
-    <workbookView xWindow="15705" yWindow="3945" windowWidth="32145" windowHeight="15345" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start here" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3974" uniqueCount="2323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3982" uniqueCount="2326">
   <si>
     <t>Beelzebub v0.136 — ability test plan</t>
   </si>
@@ -8131,6 +8131,15 @@
   </si>
   <si>
     <t>Doesn't drop from this unit by default. `.beelz admin ability AB_Wolf_Boss_DashAttack_Double_AbilityGroup` shows enabled=off. Re-enable with `.beelz admin ability AB_Wolf_Boss_DashAttack_Double_AbilityGroup enabled true`.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Works with 120 second cooldown </t>
+  </si>
+  <si>
+    <t>Works with 3 sec shortened cooldown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Works with 10 second cooldown.  However, notably there are two of this ability.  Only one gained the cooldown.  Also notably the other without the cooldown is a chain attack.  There are two attacks in the series, each of which is triggered via button push.  I don't know if the one with a cooldown was the same.  </t>
   </si>
 </sst>
 </file>
@@ -8841,7 +8850,7 @@
       </c>
       <c r="C6" s="6">
         <f>COUNTIF(Presets!L2:L210,"Pass")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D6" s="7">
         <f>COUNTIF(Presets!L2:L210,"Partial")</f>
@@ -8857,7 +8866,7 @@
       </c>
       <c r="G6" s="10">
         <f>IF(B6=0,0,SUM(C6:F6)/B6)</f>
-        <v>0</v>
+        <v>1.9138755980861243E-2</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -8926,7 +8935,7 @@
       </c>
       <c r="C9" s="13">
         <f>SUM(C6:C8)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D9" s="14">
         <f>SUM(D6:D8)</f>
@@ -8942,7 +8951,7 @@
       </c>
       <c r="G9" s="10">
         <f>IF(B9=0,0,SUM(C9:F9)/B9)</f>
-        <v>0</v>
+        <v>6.5040650406504065E-3</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
@@ -9255,8 +9264,12 @@
       <c r="J2" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="K2" s="20"/>
-      <c r="L2" s="21"/>
+      <c r="K2" s="20" t="s">
+        <v>2323</v>
+      </c>
+      <c r="L2" s="21" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" spans="1:12" ht="78.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
@@ -9289,8 +9302,12 @@
       <c r="J3" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="21"/>
+      <c r="K3" s="20" t="s">
+        <v>2323</v>
+      </c>
+      <c r="L3" s="21" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" spans="1:12" ht="78.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
@@ -9323,8 +9340,12 @@
       <c r="J4" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="K4" s="20"/>
-      <c r="L4" s="21"/>
+      <c r="K4" s="20" t="s">
+        <v>2324</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" spans="1:12" ht="108.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
@@ -9357,8 +9378,12 @@
       <c r="J5" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="K5" s="20"/>
-      <c r="L5" s="21"/>
+      <c r="K5" s="20" t="s">
+        <v>2325</v>
+      </c>
+      <c r="L5" s="21" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="6" spans="1:12" ht="78.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5">

</xml_diff>